<commit_message>
Add new funct - OBS Mat Request
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/OBSMatReq Template.xlsx
+++ b/bin/Debug/Template/OBSMatReq Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RACHHAN-PC\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2. My Project\C#\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28836927-C8B4-4575-85B3-544942186590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D8BE8D-0E6C-453D-9BBB-921B64055D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{0D9FBBC9-0A6C-4B94-8F22-EFA4A622CCA8}"/>
+    <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="15720" xr2:uid="{0D9FBBC9-0A6C-4B94-8F22-EFA4A622CCA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Rachhan System" sheetId="2" r:id="rId1"/>
@@ -25,6 +25,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -108,7 +117,7 @@
     <numFmt numFmtId="164" formatCode="0000"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy\ hh:mm\ AM/PM"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -229,6 +238,13 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Kh Battambang"/>
     </font>
   </fonts>
   <fills count="3">
@@ -449,107 +465,107 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="11" fillId="0" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="6" fillId="0" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="11" fillId="0" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="6" fillId="0" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="18" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -900,108 +916,108 @@
       <c r="F1" s="42"/>
       <c r="G1" s="42"/>
       <c r="H1" s="42"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
     </row>
     <row r="2" spans="1:11" ht="44.25" customHeight="1" thickBot="1">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="39" t="s">
+      <c r="B2" s="31"/>
+      <c r="C2" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="39" t="s">
+      <c r="F2" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="38" t="s">
+      <c r="G2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="37"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
     </row>
-    <row r="3" spans="1:11" s="30" customFormat="1" ht="39.950000000000003" customHeight="1">
-      <c r="A3" s="35" t="s">
+    <row r="3" spans="1:11" s="22" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A3" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="31" t="s">
+      <c r="H3" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="22"/>
+      <c r="I3" s="14"/>
     </row>
-    <row r="4" spans="1:11" s="21" customFormat="1" ht="65.099999999999994" customHeight="1">
-      <c r="A4" s="29"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="23" t="str">
+    <row r="4" spans="1:11" s="13" customFormat="1" ht="65.099999999999994" customHeight="1">
+      <c r="A4" s="21"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="15" t="str">
         <f>"*"&amp;A4&amp;G4&amp;"*"</f>
         <v>**</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="14" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="42" thickBot="1">
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="H5" s="19"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="H5" s="11"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="35.25" customHeight="1">
-      <c r="C7" s="15"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="12"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" spans="1:11" ht="42" thickBot="1">
-      <c r="C8" s="11"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="8"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="41"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>